<commit_message>
Update prepush data and records
</commit_message>
<xml_diff>
--- a/推免填报记录表-勾选版.xlsx
+++ b/推免填报记录表-勾选版.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,44 +28,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Microsoft YaHei"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-    </font>
-    <font>
-      <name val="Microsoft YaHei"/>
-      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001F4E78"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E7E6E6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E2F0D9"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -73,30 +47,16 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <bottom style="thin">
-        <color rgb="00D9E2F3"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -467,16 +427,16 @@
   <dimension ref="A1:J57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="48" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="46" customWidth="1" min="9" max="9"/>
-    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -531,7 +491,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42" customHeight="1">
+    <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>北京大学</t>
@@ -550,7 +510,7 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="2" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -563,7 +523,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="42" customHeight="1">
+    <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>北京航空航天大学</t>
@@ -582,7 +542,7 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -595,7 +555,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="42" customHeight="1">
+    <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>北京交通大学</t>
@@ -618,7 +578,7 @@
           <t>计算机科学与技术学院</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
@@ -631,11 +591,11 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="42" customHeight="1">
+          <t>本次未定位到2027学院原文，只保留往年学院办法作材料准备参考。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>北京科技大学</t>
@@ -658,7 +618,7 @@
           <t>计算机与通信工程学院</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>已截止</t>
         </is>
@@ -675,11 +635,11 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="42" customHeight="1">
+          <t>学院官方通知明确即日起至2026-08-30 23:59；8月31已截止，但信息完整，可用于核对后续正式推免。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>北京理工大学</t>
@@ -698,7 +658,7 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="2" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -711,7 +671,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="42" customHeight="1">
+    <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>北京师范大学</t>
@@ -730,7 +690,7 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -743,7 +703,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="42" customHeight="1">
+    <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>北京邮电大学</t>
@@ -766,7 +726,7 @@
           <t>计算机学院（国家示范性软件学院）；网络空间安全学院；人工智能学院</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>正在报名</t>
         </is>
@@ -783,11 +743,11 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="42" customHeight="1">
+          <t>北邮研招官方汇总列出人工智能学院2027实施细则入口。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
           <t>重庆大学</t>
@@ -810,7 +770,7 @@
           <t>计算机学院、软件学院、大数据与软件学院等计算机相关单位</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>正在报名</t>
         </is>
@@ -827,11 +787,11 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="42" customHeight="1">
+          <t>校级官方预报名系统开放至2026-09-30 18:00；各学院具体起止时间以系统和学院通知为准。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>大连理工大学</t>
@@ -854,7 +814,7 @@
           <t>计算机科学与技术学院；人工智能学院；软件学院（开发区校区）</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>正在报名</t>
         </is>
@@ -871,11 +831,11 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="42" customHeight="1">
+          <t>大连理工官方汇总已列出计算机科学与技术学院时间：2026-07-13 09:00至2026-09-07 09:00。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t>电子科技大学</t>
@@ -894,7 +854,7 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="2" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -907,7 +867,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="42" customHeight="1">
+    <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>东北大学</t>
@@ -930,7 +890,7 @@
           <t>计算机科学与工程学院/软件学院等</t>
         </is>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
@@ -943,11 +903,11 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="42" customHeight="1">
+          <t>校级办法已出，学院截止时间需进系统或学院通知确认。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
           <t>东南大学</t>
@@ -970,7 +930,7 @@
           <t>计算机科学与工程学院、软件学院；网络空间安全学院；雷恩研究生学院</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>已截止</t>
         </is>
@@ -987,11 +947,11 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="42" customHeight="1">
+          <t>计算机学院通知列表已发布雷恩研究生学院计算机技术专业2027推免报名通知。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>复旦大学</t>
@@ -1014,7 +974,7 @@
           <t>研究生院/计算机相关院系</t>
         </is>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
@@ -1027,11 +987,11 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="42" customHeight="1">
+          <t>学校级入口已定位，计算机相关院系原文与截止时间需在系统内继续核验。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>国防科技大学</t>
@@ -1054,7 +1014,7 @@
           <t>计算机学院、智能科学学院等</t>
         </is>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
@@ -1067,11 +1027,11 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="42" customHeight="1">
+          <t>学校方案明确有意申报2027级推免必须先通过国防科大报名系统预报名；只写7月-9月，未给统一截止日，需进系统和联系学院确认。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>哈尔滨工程大学</t>
@@ -1094,7 +1054,7 @@
           <t>计算机科学与技术学院</t>
         </is>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
@@ -1107,11 +1067,11 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="42" customHeight="1">
+          <t>学院官网标题确认是2027预报名前信息发布，但正文未稳定公开提取；先列待复核，避免误导。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>哈尔滨工业大学</t>
@@ -1134,7 +1094,7 @@
           <t>计算学部</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>已截止</t>
         </is>
@@ -1151,11 +1111,11 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="42" customHeight="1">
+          <t>已截止。计算学部和你的 CS 背景高度匹配，后续正式推免系统开放时仍可关注是否补录/追加通知。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>合肥工业大学</t>
@@ -1178,7 +1138,7 @@
           <t>计算机与信息学院（人工智能学院）等</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>正在报名</t>
         </is>
@@ -1195,11 +1155,11 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="42" customHeight="1">
+          <t>校级官方通知明确 2026-08-26 09:00 至 2026-09-15 17:00；计算机与信息学院需继续关注学院复试安排。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
           <t>河海大学</t>
@@ -1222,7 +1182,7 @@
           <t>计算机与软件学院、人工智能与自动化学院</t>
         </is>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
@@ -1235,11 +1195,11 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="42" customHeight="1">
+          <t>官方公告正文抓取很少，不能写死截止时间；列入待复核但保留入口。</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>湖南大学</t>
@@ -1262,7 +1222,7 @@
           <t>计算机学院</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
@@ -1275,11 +1235,11 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="42" customHeight="1">
+          <t>学院官方通知已发布，8月28日后可在湖南大学接收推免生报名信息采集系统提交；学院未写固定截止日，需进系统确认。</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
           <t>华北电力大学</t>
@@ -1298,7 +1258,7 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="2" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -1311,7 +1271,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="42" customHeight="1">
+    <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
           <t>华东师范大学</t>
@@ -1334,7 +1294,7 @@
           <t>计算机科学与技术学院；信息与电子工程学院（集成电路科学与工程学院）</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>正在报名</t>
         </is>
@@ -1351,11 +1311,11 @@
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="42" customHeight="1">
+          <t>官方页已发布但抓取正文不稳定；截止时间来自同批汇总线索，填报前进系统再确认。</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
           <t>华中科技大学</t>
@@ -1374,7 +1334,7 @@
       <c r="D23" s="2" t="inlineStr"/>
       <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -1387,7 +1347,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="42" customHeight="1">
+    <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
           <t>吉林大学</t>
@@ -1406,7 +1366,7 @@
       <c r="D24" s="2" t="inlineStr"/>
       <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -1419,7 +1379,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="42" customHeight="1">
+    <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
           <t>兰州大学</t>
@@ -1438,7 +1398,7 @@
       <c r="D25" s="2" t="inlineStr"/>
       <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -1451,7 +1411,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="42" customHeight="1">
+    <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
           <t>南方科技大学</t>
@@ -1474,9 +1434,9 @@
           <t>计算机科学与工程系</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr">
-        <is>
-          <t>正在报名</t>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>已截止</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
@@ -1491,11 +1451,11 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="42" customHeight="1">
+          <t>官方计算机系通知明确计算机大类含计算机科学与技术、软件工程、网安、人工智能、智能科学与技术；作为强计算机/AI补充项列入双一流补充。</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
           <t>南京大学</t>
@@ -1518,7 +1478,7 @@
           <t>软件学院；智能软件与工程学院</t>
         </is>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
@@ -1531,11 +1491,11 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="42" customHeight="1">
+          <t>苏州校区智能软件与工程学院单独发布通知，适合软件/AI方向补充关注。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
           <t>南京航空航天大学</t>
@@ -1558,7 +1518,7 @@
           <t>计算机科学与技术学院/人工智能学院等</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>正在报名</t>
         </is>
@@ -1575,11 +1535,11 @@
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="42" customHeight="1">
+          <t>校级系统已开，需重点查计算机学院是否有早截止。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
           <t>南京理工大学</t>
@@ -1602,9 +1562,9 @@
           <t>计算机科学与工程学院（人工智能学院、软件学院）</t>
         </is>
       </c>
-      <c r="G29" s="5" t="inlineStr">
-        <is>
-          <t>正在报名</t>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>已截止</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -1619,11 +1579,11 @@
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="42" customHeight="1">
+          <t>2027计算机学院具体内容目前主要通过学校预推免入口和聚合线索定位，填报前务必复核学院原文。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
           <t>南开大学</t>
@@ -1646,7 +1606,7 @@
           <t>计算机学院、密码与网络空间安全学院；软件学院</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>正在报名</t>
         </is>
@@ -1663,11 +1623,11 @@
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="42" customHeight="1">
+          <t>官方学院通知明确报名至2026-09-12；要求先联系导师/实验室，别只填系统。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
           <t>清华大学</t>
@@ -1690,7 +1650,7 @@
           <t>研究生院/计算机科学与技术系/深圳国际研究生院</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>已截止</t>
         </is>
@@ -1707,11 +1667,11 @@
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="42" customHeight="1">
+          <t>已截止。清华 CS 系主要看到直博简章，硕士方向以系统和目录为准。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
           <t>厦门大学</t>
@@ -1734,7 +1694,7 @@
           <t>信息学院（特色化示范性软件学院）</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>已截止</t>
         </is>
@@ -1751,11 +1711,11 @@
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="42" customHeight="1">
+          <t>已截止，但材料要求很完整，可作为其他学校材料准备模板。</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
           <t>山东大学</t>
@@ -1778,7 +1738,7 @@
           <t>计算机科学与技术学院、软件学院、人工智能学院等</t>
         </is>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
@@ -1791,11 +1751,11 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="42" customHeight="1">
+          <t>校级系统 2026-09-01 09:00 开放；每名考生最多选择三个招生单位，每个招生单位一个专业，报名期内可修改后重新提交。</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
           <t>上海大学</t>
@@ -1814,7 +1774,7 @@
       <c r="D34" s="2" t="inlineStr"/>
       <c r="E34" s="2" t="inlineStr"/>
       <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -1827,7 +1787,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="42" customHeight="1">
+    <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
           <t>上海交通大学</t>
@@ -1846,7 +1806,7 @@
       <c r="D35" s="2" t="inlineStr"/>
       <c r="E35" s="2" t="inlineStr"/>
       <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -1859,7 +1819,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="42" customHeight="1">
+    <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
           <t>四川大学</t>
@@ -1878,7 +1838,7 @@
       <c r="D36" s="2" t="inlineStr"/>
       <c r="E36" s="2" t="inlineStr"/>
       <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -1891,7 +1851,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="42" customHeight="1">
+    <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
           <t>苏州大学</t>
@@ -1914,7 +1874,7 @@
           <t>计算机科学与技术学院</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>已截止</t>
         </is>
@@ -1931,11 +1891,11 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="42" customHeight="1">
+          <t>学院官方通知明确系统暂定开放 2026-08-15 至 2026-08-28；已截止，但考核安排和“不可修改”很关键。</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
           <t>天津大学</t>
@@ -1958,7 +1918,7 @@
           <t>智能与计算学部等计算机相关单位</t>
         </is>
       </c>
-      <c r="G38" s="5" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>正在报名</t>
         </is>
@@ -1975,11 +1935,11 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="42" customHeight="1">
+          <t>学校系统已开，智能与计算学部细则需在学院网站继续看。</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
           <t>同济大学</t>
@@ -2002,7 +1962,7 @@
           <t>计算机科学与技术学院（软件学院）</t>
         </is>
       </c>
-      <c r="G39" s="4" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>已截止</t>
         </is>
@@ -2019,11 +1979,11 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="42" customHeight="1">
+          <t>研招网汇总明确该学院截止 2026-08-25 12:00。</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
           <t>武汉大学</t>
@@ -2042,7 +2002,7 @@
       <c r="D40" s="2" t="inlineStr"/>
       <c r="E40" s="2" t="inlineStr"/>
       <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -2055,7 +2015,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="42" customHeight="1">
+    <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
           <t>武汉理工大学</t>
@@ -2074,7 +2034,7 @@
       <c r="D41" s="2" t="inlineStr"/>
       <c r="E41" s="2" t="inlineStr"/>
       <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" s="3" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -2087,7 +2047,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="42" customHeight="1">
+    <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
           <t>西安电子科技大学</t>
@@ -2110,7 +2070,7 @@
           <t>计算机科学与技术学院（国家示范性软件学院）；人工智能学院</t>
         </is>
       </c>
-      <c r="G42" s="5" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>正在报名</t>
         </is>
@@ -2127,11 +2087,11 @@
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="42" customHeight="1">
+          <t>学院官方2027推荐免试研究生招生预报名通知；仅可选择一个学院预报名，正式录取仍须通过中国研招网推免服务系统。</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
           <t>西安交通大学</t>
@@ -2150,7 +2110,7 @@
       <c r="D43" s="2" t="inlineStr"/>
       <c r="E43" s="2" t="inlineStr"/>
       <c r="F43" s="2" t="inlineStr"/>
-      <c r="G43" s="3" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -2163,7 +2123,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="42" customHeight="1">
+    <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
           <t>西北工业大学</t>
@@ -2182,7 +2142,7 @@
       <c r="D44" s="2" t="inlineStr"/>
       <c r="E44" s="2" t="inlineStr"/>
       <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="3" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -2195,7 +2155,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="42" customHeight="1">
+    <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
           <t>西北农林科技大学</t>
@@ -2214,7 +2174,7 @@
       <c r="D45" s="2" t="inlineStr"/>
       <c r="E45" s="2" t="inlineStr"/>
       <c r="F45" s="2" t="inlineStr"/>
-      <c r="G45" s="3" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -2227,7 +2187,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="42" customHeight="1">
+    <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
           <t>西南财经大学</t>
@@ -2250,9 +2210,9 @@
           <t>计算机与人工智能学院</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr">
-        <is>
-          <t>正在报名</t>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>已截止</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -2267,11 +2227,11 @@
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="42" customHeight="1">
+          <t>中上游211补充项，学院官方明确计算机科学与技术和电子信息两个专业，报名期至2026-08-31。</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
           <t>西南交通大学</t>
@@ -2290,7 +2250,7 @@
       <c r="D47" s="2" t="inlineStr"/>
       <c r="E47" s="2" t="inlineStr"/>
       <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="3" t="inlineStr">
+      <c r="G47" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -2303,7 +2263,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="42" customHeight="1">
+    <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
           <t>浙江大学</t>
@@ -2326,7 +2286,7 @@
           <t>计算机科学与技术学院；人工智能学院</t>
         </is>
       </c>
-      <c r="G48" s="5" t="inlineStr">
+      <c r="G48" s="2" t="inlineStr">
         <is>
           <t>正在报名</t>
         </is>
@@ -2343,11 +2303,11 @@
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="42" customHeight="1">
+          <t>学院官方通知明确 2026-08-10 09:00 至 2026-09-10 24:00；每人只能填报一个志愿，计算机背景报AI方向可重点看。</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
           <t>郑州大学</t>
@@ -2366,7 +2326,7 @@
       <c r="D49" s="2" t="inlineStr"/>
       <c r="E49" s="2" t="inlineStr"/>
       <c r="F49" s="2" t="inlineStr"/>
-      <c r="G49" s="3" t="inlineStr">
+      <c r="G49" s="2" t="inlineStr">
         <is>
           <t>未定位</t>
         </is>
@@ -2379,7 +2339,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="42" customHeight="1">
+    <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
           <t>中国海洋大学</t>
@@ -2402,7 +2362,7 @@
           <t>信息科学与工程学部等计算机相关单位</t>
         </is>
       </c>
-      <c r="G50" s="5" t="inlineStr">
+      <c r="G50" s="2" t="inlineStr">
         <is>
           <t>正在报名</t>
         </is>
@@ -2419,11 +2379,11 @@
       </c>
       <c r="J50" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="42" customHeight="1">
+          <t>研招办官方通知明确预报名 2026-07-23 至 2026-09-14 17:00；硕士报名和直博报名最多可分别填三个不同志愿。</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
           <t>中国科学技术大学</t>
@@ -2446,24 +2406,28 @@
           <t>计算机科学与技术学院；网络空间安全学院；人工智能与数据科学学院</t>
         </is>
       </c>
-      <c r="G51" s="3" t="inlineStr">
-        <is>
-          <t>待复核</t>
-        </is>
-      </c>
-      <c r="H51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>正在报名</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>https://yjszs.ustc.edu.cn</t>
+          <t>https://xspt.ustc.edu.cn/</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="42" customHeight="1">
+          <t>8月31日最新官方预面试报名通知，9月9日截止；这是当前最值得优先看的中科大AI/数据方向入口。</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
           <t>中国矿业大学</t>
@@ -2486,7 +2450,7 @@
           <t>计算机科学与技术学院、人工智能相关专项等</t>
         </is>
       </c>
-      <c r="G52" s="5" t="inlineStr">
+      <c r="G52" s="2" t="inlineStr">
         <is>
           <t>正在报名</t>
         </is>
@@ -2503,11 +2467,11 @@
       </c>
       <c r="J52" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="42" customHeight="1">
+          <t>学校官方预报名系统 2026-08-20 至 2026-09-18 17:00 开放；人工智能拔尖创新人才专项可在系统中选择。</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
           <t>中国农业大学</t>
@@ -2530,9 +2494,9 @@
           <t>信息与电气工程学院等计算机/人工智能相关单位</t>
         </is>
       </c>
-      <c r="G53" s="5" t="inlineStr">
-        <is>
-          <t>正在报名</t>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>已截止</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -2547,11 +2511,11 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="42" customHeight="1">
+          <t>研招办发布2027各院系接收推免工作实施细则汇总，信息与电气工程学院在汇总列表中；学院原文需继续复核。</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
           <t>中国人民大学</t>
@@ -2574,7 +2538,7 @@
           <t>高瓴人工智能学院</t>
         </is>
       </c>
-      <c r="G54" s="4" t="inlineStr">
+      <c r="G54" s="2" t="inlineStr">
         <is>
           <t>已截止</t>
         </is>
@@ -2591,11 +2555,11 @@
       </c>
       <c r="J54" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="42" customHeight="1">
+          <t>官方学院通知明确2027年推免生接收报名；已截止，但AI方向和材料要求值得参考。</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
           <t>中南大学</t>
@@ -2618,7 +2582,7 @@
           <t>计算机学院/自动化学院/大数据研究院等计算机相关单位</t>
         </is>
       </c>
-      <c r="G55" s="3" t="inlineStr">
+      <c r="G55" s="2" t="inlineStr">
         <is>
           <t>待复核</t>
         </is>
@@ -2631,11 +2595,11 @@
       </c>
       <c r="J55" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="42" customHeight="1">
+          <t>校级官方预报名8月28日开始，各二级单位截止时间不同；填计算机类前必须再看对应学院通知。</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
           <t>中山大学</t>
@@ -2658,7 +2622,7 @@
           <t>计算机学院；网络空间安全学院</t>
         </is>
       </c>
-      <c r="G56" s="4" t="inlineStr">
+      <c r="G56" s="2" t="inlineStr">
         <is>
           <t>已截止</t>
         </is>
@@ -2675,11 +2639,11 @@
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="42" customHeight="1">
+          <t>要求具体，动作多，建议尽早准备视频和测评。</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
           <t>中央民族大学</t>
@@ -2702,7 +2666,7 @@
           <t>信息工程学院</t>
         </is>
       </c>
-      <c r="G57" s="4" t="inlineStr">
+      <c r="G57" s="2" t="inlineStr">
         <is>
           <t>已截止</t>
         </is>
@@ -2719,20 +2683,12 @@
       </c>
       <c r="J57" s="2" t="inlineStr">
         <is>
-          <t>按网站卡片逐项核对学院通知，填写后可在本表改为☑ 是。</t>
+          <t>学院官方通知明确 2026-08-01 00:00 至 2026-08-18 17:00，已截止；复试时间和材料要求完整保留。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J57"/>
-  <dataValidations count="2">
-    <dataValidation sqref="B2:B57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"☑ 是,☐ 否"</formula1>
-    </dataValidation>
-    <dataValidation sqref="C2:C57" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"可修改,不可修改,待确认"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>